<commit_message>
Added course booking popup and course UI updates
</commit_message>
<xml_diff>
--- a/service_bookings.xlsx
+++ b/service_bookings.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F8"/>
+  <dimension ref="A1:F10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -642,6 +642,60 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>dhanusha</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>dhanusha.selvaraj05@gmail.com</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>09344520475</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Dynamic Websites</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>hi</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>dhanusha</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>dhanusha.selvaraj05@gmail.com</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>09344520475</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Dynamic Websites</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>hi</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Updated service page UI and dropdown improvements
</commit_message>
<xml_diff>
--- a/service_bookings.xlsx
+++ b/service_bookings.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F29"/>
+  <dimension ref="A1:F30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1123,7 +1123,29 @@
           <t>CRM projects</t>
         </is>
       </c>
-      <c r="F29" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>dhanusha</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>dhanusha.selvaraj05@gmail.com</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>9344520475</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Dynamic Websites</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>